<commit_message>
Add a number-format display layer
Cells now render through their number format while editing the raw value:
- .xlsx: resolve the cell's format code from xl/styles.xml (custom numFmts +
  built-in ids) and apply it with SSF (bundled with the formula engine).
- .ods: use the producer's formatted text from <text:p> as the display.
Typed values keep the cell's format and recomputed formula results are
re-formatted. The grid shows the formatted text; focusing a cell reveals the
raw value (or the formula) for editing.

Covered by vitest (date/currency/General + recompute + ods) and a Cypress
display-layer e2e.
</commit_message>
<xml_diff>
--- a/cypress/fixtures/sample.xlsx
+++ b/cypress/fixtures/sample.xlsx
@@ -5,6 +5,18 @@
     <sheet name="Budget" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+  </numFmts>
+  <cellXfs count="2">
+    <xf numFmtId="0"/>
+    <xf numFmtId="164"/>
+  </cellXfs>
+</styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -26,6 +38,11 @@
           <t>total</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -40,6 +57,9 @@
         <f>B2*2</f>
         <v>6</v>
       </c>
+      <c r="D2" s="1">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -53,6 +73,9 @@
       <c r="C3">
         <f>B3*2</f>
         <v>8</v>
+      </c>
+      <c r="D3" s="1">
+        <v>4.25</v>
       </c>
     </row>
     <row r="4">

</xml_diff>